<commit_message>
Add baseline emission factors for China's regional power grids for 2016-2022
- Introduced new Excel file C_Control_Variable.xlsx for control variable data.
- Added PDF documents detailing baseline emission factors for the years 2016, 2017, 2019, 2021, and 2022, including methodologies and results.
- Included regional breakdowns and calculations for marginal emission factors (OM and BM) for various power grids across China.
- Ensured all documents follow the latest CDM guidelines and reflect accurate data for stakeholders.
</commit_message>
<xml_diff>
--- a/Data/C_Control_Variable.xlsx
+++ b/Data/C_Control_Variable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\statistical-model\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B2960FF-D61B-4B21-9D4F-408FE6B3F498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B7A04D-2697-4F3F-B465-91AE521A5927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="33">
   <si>
     <t>province_code</t>
   </si>
@@ -132,13 +132,29 @@
   <si>
     <t>聚金数据，上海有色网</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2023 年电力二氧化碳排放因子</t>
+  </si>
+  <si>
+    <t>关于发布2022年电力二氧化碳排放因子的公告</t>
+  </si>
+  <si>
+    <t>2021年电力二氧化碳排放因子</t>
+  </si>
+  <si>
+    <t>海东市“十三五”控制温室气体排放目标责任考核实施方案</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中国区域电网二氧化碳排放因子研究（2023）</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,6 +164,14 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -189,12 +213,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -482,7 +507,7 @@
     <col min="5" max="5" width="12.77734375" customWidth="1"/>
     <col min="7" max="7" width="15.77734375" customWidth="1"/>
     <col min="8" max="8" width="18.88671875" customWidth="1"/>
-    <col min="9" max="9" width="45.6640625" customWidth="1"/>
+    <col min="9" max="9" width="49.77734375" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
     <col min="11" max="11" width="22.44140625" customWidth="1"/>
     <col min="12" max="12" width="24.5546875" customWidth="1"/>
@@ -538,6 +563,9 @@
       <c r="C2">
         <v>0.51490000000000002</v>
       </c>
+      <c r="D2">
+        <v>0.1116</v>
+      </c>
       <c r="F2" s="2">
         <v>12206</v>
       </c>
@@ -546,6 +574,9 @@
       </c>
       <c r="H2" t="s">
         <v>11</v>
+      </c>
+      <c r="I2" t="s">
+        <v>31</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
@@ -616,6 +647,9 @@
       <c r="C5">
         <v>0.51149999999999995</v>
       </c>
+      <c r="D5">
+        <v>9.1999999999999998E-2</v>
+      </c>
       <c r="F5" s="2">
         <v>14293</v>
       </c>
@@ -624,6 +658,9 @@
       </c>
       <c r="H5" t="s">
         <v>11</v>
+      </c>
+      <c r="I5" t="s">
+        <v>32</v>
       </c>
       <c r="K5" t="s">
         <v>27</v>
@@ -669,7 +706,7 @@
         <v>0.51449999999999996</v>
       </c>
       <c r="D7">
-        <v>1.48</v>
+        <v>0.14799999999999999</v>
       </c>
       <c r="F7" s="2">
         <v>14101</v>
@@ -700,6 +737,9 @@
       <c r="C8">
         <v>0.52359999999999995</v>
       </c>
+      <c r="D8">
+        <v>0.1235</v>
+      </c>
       <c r="F8" s="2">
         <v>18923</v>
       </c>
@@ -708,6 +748,9 @@
       </c>
       <c r="H8" t="s">
         <v>11</v>
+      </c>
+      <c r="I8" t="s">
+        <v>30</v>
       </c>
       <c r="K8" t="s">
         <v>27</v>
@@ -726,6 +769,9 @@
       <c r="C9">
         <v>0.52980000000000005</v>
       </c>
+      <c r="D9" s="3">
+        <v>0.10730000000000001</v>
+      </c>
       <c r="F9" s="2">
         <v>19929</v>
       </c>
@@ -734,6 +780,9 @@
       </c>
       <c r="H9" t="s">
         <v>11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>29</v>
       </c>
       <c r="K9" t="s">
         <v>27</v>
@@ -752,6 +801,9 @@
       <c r="C10">
         <v>0.53520000000000001</v>
       </c>
+      <c r="D10">
+        <v>0.1333</v>
+      </c>
       <c r="F10" s="2">
         <v>18687</v>
       </c>
@@ -760,6 +812,9 @@
       </c>
       <c r="H10" t="s">
         <v>11</v>
+      </c>
+      <c r="I10" t="s">
+        <v>28</v>
       </c>
       <c r="K10" t="s">
         <v>27</v>
@@ -830,6 +885,9 @@
       <c r="C13">
         <v>0.51400000000000001</v>
       </c>
+      <c r="D13">
+        <v>0.35730000000000001</v>
+      </c>
       <c r="F13" s="2">
         <v>12206</v>
       </c>
@@ -838,6 +896,9 @@
       </c>
       <c r="H13" t="s">
         <v>11</v>
+      </c>
+      <c r="I13" t="s">
+        <v>31</v>
       </c>
       <c r="K13" t="s">
         <v>27</v>
@@ -908,6 +969,9 @@
       <c r="C16">
         <v>0.51129999999999998</v>
       </c>
+      <c r="D16">
+        <v>0.39400000000000002</v>
+      </c>
       <c r="F16" s="2">
         <v>14293</v>
       </c>
@@ -916,6 +980,9 @@
       </c>
       <c r="H16" t="s">
         <v>11</v>
+      </c>
+      <c r="I16" t="s">
+        <v>32</v>
       </c>
       <c r="K16" t="s">
         <v>27</v>
@@ -961,7 +1028,7 @@
         <v>0.51400000000000001</v>
       </c>
       <c r="D18">
-        <v>5.18</v>
+        <v>0.51800000000000002</v>
       </c>
       <c r="F18" s="2">
         <v>14101</v>
@@ -992,6 +1059,9 @@
       <c r="C19">
         <v>0.52349999999999997</v>
       </c>
+      <c r="D19">
+        <v>0.51539999999999997</v>
+      </c>
       <c r="F19" s="2">
         <v>18923</v>
       </c>
@@ -1000,6 +1070,9 @@
       </c>
       <c r="H19" t="s">
         <v>11</v>
+      </c>
+      <c r="I19" t="s">
+        <v>30</v>
       </c>
       <c r="K19" t="s">
         <v>27</v>
@@ -1018,6 +1091,9 @@
       <c r="C20">
         <v>0.53</v>
       </c>
+      <c r="D20" s="3">
+        <v>0.40439999999999998</v>
+      </c>
       <c r="F20" s="2">
         <v>19929</v>
       </c>
@@ -1026,6 +1102,9 @@
       </c>
       <c r="H20" t="s">
         <v>11</v>
+      </c>
+      <c r="I20" t="s">
+        <v>29</v>
       </c>
       <c r="K20" t="s">
         <v>27</v>
@@ -1044,6 +1123,9 @@
       <c r="C21">
         <v>0.53600000000000003</v>
       </c>
+      <c r="D21">
+        <v>0.4476</v>
+      </c>
       <c r="F21" s="2">
         <v>18687</v>
       </c>
@@ -1052,6 +1134,9 @@
       </c>
       <c r="H21" t="s">
         <v>11</v>
+      </c>
+      <c r="I21" t="s">
+        <v>28</v>
       </c>
       <c r="K21" t="s">
         <v>27</v>
@@ -1122,6 +1207,9 @@
       <c r="C24">
         <v>0.39889999999999998</v>
       </c>
+      <c r="D24">
+        <v>0.79390000000000005</v>
+      </c>
       <c r="F24" s="2">
         <v>12206</v>
       </c>
@@ -1130,6 +1218,9 @@
       </c>
       <c r="H24" t="s">
         <v>11</v>
+      </c>
+      <c r="I24" t="s">
+        <v>31</v>
       </c>
       <c r="K24" t="s">
         <v>27</v>
@@ -1200,6 +1291,9 @@
       <c r="C27">
         <v>0.40210000000000001</v>
       </c>
+      <c r="D27">
+        <v>0.753</v>
+      </c>
       <c r="F27" s="2">
         <v>14293</v>
       </c>
@@ -1208,6 +1302,9 @@
       </c>
       <c r="H27" t="s">
         <v>11</v>
+      </c>
+      <c r="I27" t="s">
+        <v>32</v>
       </c>
       <c r="K27" t="s">
         <v>27</v>
@@ -1253,7 +1350,7 @@
         <v>0.40379999999999999</v>
       </c>
       <c r="D29">
-        <v>10.49</v>
+        <v>1.0489999999999999</v>
       </c>
       <c r="F29" s="2">
         <v>14101</v>
@@ -1284,6 +1381,9 @@
       <c r="C30">
         <v>0.40389999999999998</v>
       </c>
+      <c r="D30">
+        <v>0.70250000000000001</v>
+      </c>
       <c r="F30" s="2">
         <v>18923</v>
       </c>
@@ -1292,6 +1392,9 @@
       </c>
       <c r="H30" t="s">
         <v>11</v>
+      </c>
+      <c r="I30" t="s">
+        <v>30</v>
       </c>
       <c r="K30" t="s">
         <v>27</v>
@@ -1310,6 +1413,9 @@
       <c r="C31">
         <v>0.4042</v>
       </c>
+      <c r="D31" s="3">
+        <v>0.68489999999999995</v>
+      </c>
       <c r="F31" s="2">
         <v>19929</v>
       </c>
@@ -1318,6 +1424,9 @@
       </c>
       <c r="H31" t="s">
         <v>11</v>
+      </c>
+      <c r="I31" t="s">
+        <v>29</v>
       </c>
       <c r="K31" t="s">
         <v>27</v>
@@ -1336,6 +1445,9 @@
       <c r="C32">
         <v>0.40450000000000003</v>
       </c>
+      <c r="D32">
+        <v>0.64790000000000003</v>
+      </c>
       <c r="F32" s="2">
         <v>18687</v>
       </c>
@@ -1344,6 +1456,9 @@
       </c>
       <c r="H32" t="s">
         <v>11</v>
+      </c>
+      <c r="I32" t="s">
+        <v>28</v>
       </c>
       <c r="K32" t="s">
         <v>27</v>
@@ -1414,6 +1529,9 @@
       <c r="C35">
         <v>0.74670000000000003</v>
       </c>
+      <c r="D35">
+        <v>0.81159999999999999</v>
+      </c>
       <c r="F35" s="2">
         <v>12206</v>
       </c>
@@ -1422,6 +1540,9 @@
       </c>
       <c r="H35" t="s">
         <v>11</v>
+      </c>
+      <c r="I35" t="s">
+        <v>31</v>
       </c>
       <c r="K35" t="s">
         <v>27</v>
@@ -1492,6 +1613,9 @@
       <c r="C38">
         <v>0.6633</v>
       </c>
+      <c r="D38">
+        <v>0.79100000000000004</v>
+      </c>
       <c r="F38" s="2">
         <v>14293</v>
       </c>
@@ -1500,6 +1624,9 @@
       </c>
       <c r="H38" t="s">
         <v>11</v>
+      </c>
+      <c r="I38" t="s">
+        <v>32</v>
       </c>
       <c r="K38" t="s">
         <v>27</v>
@@ -1545,7 +1672,7 @@
         <v>0.60499999999999998</v>
       </c>
       <c r="D40">
-        <v>7.56</v>
+        <v>0.75600000000000001</v>
       </c>
       <c r="F40" s="2">
         <v>14101</v>
@@ -1576,6 +1703,9 @@
       <c r="C41">
         <v>0.6</v>
       </c>
+      <c r="D41">
+        <v>0.63690000000000002</v>
+      </c>
       <c r="F41" s="2">
         <v>18923</v>
       </c>
@@ -1584,6 +1714,9 @@
       </c>
       <c r="H41" t="s">
         <v>11</v>
+      </c>
+      <c r="I41" t="s">
+        <v>30</v>
       </c>
       <c r="K41" t="s">
         <v>27</v>
@@ -1602,6 +1735,9 @@
       <c r="C42">
         <v>0.6</v>
       </c>
+      <c r="D42" s="3">
+        <v>0.60580000000000001</v>
+      </c>
       <c r="F42" s="2">
         <v>19929</v>
       </c>
@@ -1610,6 +1746,9 @@
       </c>
       <c r="H42" t="s">
         <v>11</v>
+      </c>
+      <c r="I42" t="s">
+        <v>29</v>
       </c>
       <c r="K42" t="s">
         <v>27</v>
@@ -1628,6 +1767,9 @@
       <c r="C43">
         <v>0.6</v>
       </c>
+      <c r="D43">
+        <v>0.5897</v>
+      </c>
       <c r="F43" s="2">
         <v>18687</v>
       </c>
@@ -1636,6 +1778,9 @@
       </c>
       <c r="H43" t="s">
         <v>11</v>
+      </c>
+      <c r="I43" t="s">
+        <v>28</v>
       </c>
       <c r="K43" t="s">
         <v>27</v>
@@ -1706,6 +1851,9 @@
       <c r="C46">
         <v>0.77500000000000002</v>
       </c>
+      <c r="D46">
+        <v>0.85550000000000004</v>
+      </c>
       <c r="F46" s="2">
         <v>12206</v>
       </c>
@@ -1714,6 +1862,9 @@
       </c>
       <c r="H46" t="s">
         <v>11</v>
+      </c>
+      <c r="I46" t="s">
+        <v>31</v>
       </c>
       <c r="K46" t="s">
         <v>27</v>
@@ -1784,6 +1935,9 @@
       <c r="C49">
         <v>0.72670000000000001</v>
       </c>
+      <c r="D49">
+        <v>0.86099999999999999</v>
+      </c>
       <c r="F49" s="2">
         <v>14293</v>
       </c>
@@ -1792,6 +1946,9 @@
       </c>
       <c r="H49" t="s">
         <v>11</v>
+      </c>
+      <c r="I49" t="s">
+        <v>32</v>
       </c>
       <c r="K49" t="s">
         <v>27</v>
@@ -1837,7 +1994,7 @@
         <v>0.59750000000000003</v>
       </c>
       <c r="D51">
-        <v>7.85</v>
+        <v>0.78500000000000003</v>
       </c>
       <c r="F51" s="2">
         <v>14101</v>
@@ -1868,6 +2025,9 @@
       <c r="C52">
         <v>0.59</v>
       </c>
+      <c r="D52">
+        <v>0.68379999999999996</v>
+      </c>
       <c r="F52" s="2">
         <v>18923</v>
       </c>
@@ -1876,6 +2036,9 @@
       </c>
       <c r="H52" t="s">
         <v>11</v>
+      </c>
+      <c r="I52" t="s">
+        <v>30</v>
       </c>
       <c r="K52" t="s">
         <v>27</v>
@@ -1894,6 +2057,9 @@
       <c r="C53">
         <v>0.59</v>
       </c>
+      <c r="D53" s="3">
+        <v>0.64100000000000001</v>
+      </c>
       <c r="F53" s="2">
         <v>19929</v>
       </c>
@@ -1902,6 +2068,9 @@
       </c>
       <c r="H53" t="s">
         <v>11</v>
+      </c>
+      <c r="I53" t="s">
+        <v>29</v>
       </c>
       <c r="K53" t="s">
         <v>27</v>
@@ -1920,6 +2089,9 @@
       <c r="C54">
         <v>0.71079999999999999</v>
       </c>
+      <c r="D54">
+        <v>0.61909999999999998</v>
+      </c>
       <c r="F54" s="2">
         <v>18687</v>
       </c>
@@ -1928,6 +2100,9 @@
       </c>
       <c r="H54" t="s">
         <v>11</v>
+      </c>
+      <c r="I54" t="s">
+        <v>28</v>
       </c>
       <c r="K54" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Add new output file Y_Output.xlsx to the Data directory
</commit_message>
<xml_diff>
--- a/Data/C_Control_Variable.xlsx
+++ b/Data/C_Control_Variable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\statistical-model\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B7A04D-2697-4F3F-B465-91AE521A5927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50761E33-02C2-4E15-BC3A-C08D04E2B50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="42">
   <si>
     <t>province_code</t>
   </si>
@@ -148,6 +148,38 @@
   </si>
   <si>
     <t>中国区域电网二氧化碳排放因子研究（2023）</t>
+  </si>
+  <si>
+    <t>《中国区域电网二氧化碳排放因子研究（2016）》</t>
+  </si>
+  <si>
+    <t>《2017 年省级电网排放因子测算报告》</t>
+  </si>
+  <si>
+    <t>政策有效期内</t>
+  </si>
+  <si>
+    <t>政策有效期内</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>无产能承接政策，为产能转出省份</t>
+  </si>
+  <si>
+    <t>云南省产业发展规划（2016—2025年）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NaN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>广西铝产业二次创业中长期方案</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>内蒙古自治区规范电解铝产能置换工作的通知</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -508,7 +540,7 @@
     <col min="7" max="7" width="15.77734375" customWidth="1"/>
     <col min="8" max="8" width="18.88671875" customWidth="1"/>
     <col min="9" max="9" width="49.77734375" customWidth="1"/>
-    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="10" max="10" width="42.109375" customWidth="1"/>
     <col min="11" max="11" width="22.44140625" customWidth="1"/>
     <col min="12" max="12" width="24.5546875" customWidth="1"/>
     <col min="13" max="13" width="13.21875" customWidth="1"/>
@@ -566,6 +598,9 @@
       <c r="D2">
         <v>0.1116</v>
       </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
       <c r="F2" s="2">
         <v>12206</v>
       </c>
@@ -577,6 +612,9 @@
       </c>
       <c r="I2" t="s">
         <v>31</v>
+      </c>
+      <c r="J2" t="s">
+        <v>39</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
@@ -595,6 +633,12 @@
       <c r="C3" s="1">
         <v>0.51559999999999995</v>
       </c>
+      <c r="D3">
+        <v>0.1082</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
       <c r="F3" s="2">
         <v>12344</v>
       </c>
@@ -603,6 +647,12 @@
       </c>
       <c r="H3" t="s">
         <v>11</v>
+      </c>
+      <c r="I3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" t="s">
+        <v>38</v>
       </c>
       <c r="K3" t="s">
         <v>27</v>
@@ -621,6 +671,12 @@
       <c r="C4">
         <v>0.51370000000000005</v>
       </c>
+      <c r="D4">
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
       <c r="F4" s="2">
         <v>14631</v>
       </c>
@@ -629,6 +685,12 @@
       </c>
       <c r="H4" t="s">
         <v>11</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>35</v>
       </c>
       <c r="K4" t="s">
         <v>27</v>
@@ -650,6 +712,9 @@
       <c r="D5">
         <v>9.1999999999999998E-2</v>
       </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
       <c r="F5" s="2">
         <v>14293</v>
       </c>
@@ -661,6 +726,9 @@
       </c>
       <c r="I5" t="s">
         <v>32</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
       </c>
       <c r="K5" t="s">
         <v>27</v>
@@ -679,6 +747,12 @@
       <c r="C6">
         <v>0.5091</v>
       </c>
+      <c r="D6">
+        <v>0.10199999999999999</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
       <c r="F6" s="2">
         <v>13925</v>
       </c>
@@ -687,6 +761,9 @@
       </c>
       <c r="H6" t="s">
         <v>11</v>
+      </c>
+      <c r="J6" t="s">
+        <v>35</v>
       </c>
       <c r="K6" t="s">
         <v>27</v>
@@ -708,6 +785,9 @@
       <c r="D7">
         <v>0.14799999999999999</v>
       </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
       <c r="F7" s="2">
         <v>14101</v>
       </c>
@@ -719,6 +799,9 @@
       </c>
       <c r="I7" t="s">
         <v>25</v>
+      </c>
+      <c r="J7" t="s">
+        <v>35</v>
       </c>
       <c r="K7" t="s">
         <v>27</v>
@@ -740,6 +823,9 @@
       <c r="D8">
         <v>0.1235</v>
       </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
       <c r="F8" s="2">
         <v>18923</v>
       </c>
@@ -751,6 +837,9 @@
       </c>
       <c r="I8" t="s">
         <v>30</v>
+      </c>
+      <c r="J8" t="s">
+        <v>35</v>
       </c>
       <c r="K8" t="s">
         <v>27</v>
@@ -772,6 +861,9 @@
       <c r="D9" s="3">
         <v>0.10730000000000001</v>
       </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
       <c r="F9" s="2">
         <v>19929</v>
       </c>
@@ -783,6 +875,9 @@
       </c>
       <c r="I9" t="s">
         <v>29</v>
+      </c>
+      <c r="J9" t="s">
+        <v>35</v>
       </c>
       <c r="K9" t="s">
         <v>27</v>
@@ -804,6 +899,9 @@
       <c r="D10">
         <v>0.1333</v>
       </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
       <c r="F10" s="2">
         <v>18687</v>
       </c>
@@ -815,6 +913,9 @@
       </c>
       <c r="I10" t="s">
         <v>28</v>
+      </c>
+      <c r="J10" t="s">
+        <v>35</v>
       </c>
       <c r="K10" t="s">
         <v>27</v>
@@ -833,6 +934,12 @@
       <c r="C11">
         <v>0.54520000000000002</v>
       </c>
+      <c r="D11">
+        <v>0.129</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
       <c r="F11" s="2">
         <v>19952</v>
       </c>
@@ -841,6 +948,9 @@
       </c>
       <c r="H11" t="s">
         <v>11</v>
+      </c>
+      <c r="J11" t="s">
+        <v>35</v>
       </c>
       <c r="K11" t="s">
         <v>27</v>
@@ -859,6 +969,12 @@
       <c r="C12">
         <v>0.55059999999999998</v>
       </c>
+      <c r="D12">
+        <v>0.125</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
       <c r="F12" s="2">
         <v>20732</v>
       </c>
@@ -867,6 +983,9 @@
       </c>
       <c r="H12" t="s">
         <v>11</v>
+      </c>
+      <c r="J12" t="s">
+        <v>35</v>
       </c>
       <c r="K12" t="s">
         <v>17</v>
@@ -888,6 +1007,9 @@
       <c r="D13">
         <v>0.35730000000000001</v>
       </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
       <c r="F13" s="2">
         <v>12206</v>
       </c>
@@ -899,6 +1021,9 @@
       </c>
       <c r="I13" t="s">
         <v>31</v>
+      </c>
+      <c r="J13" t="s">
+        <v>39</v>
       </c>
       <c r="K13" t="s">
         <v>27</v>
@@ -917,6 +1042,12 @@
       <c r="C14">
         <v>0.51419999999999999</v>
       </c>
+      <c r="D14">
+        <v>0.36840000000000001</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
       <c r="F14" s="2">
         <v>12344</v>
       </c>
@@ -925,6 +1056,12 @@
       </c>
       <c r="H14" t="s">
         <v>11</v>
+      </c>
+      <c r="I14" t="s">
+        <v>33</v>
+      </c>
+      <c r="J14" t="s">
+        <v>39</v>
       </c>
       <c r="K14" t="s">
         <v>27</v>
@@ -943,6 +1080,12 @@
       <c r="C15">
         <v>0.51349999999999996</v>
       </c>
+      <c r="D15">
+        <v>0.38119999999999998</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
       <c r="F15" s="2">
         <v>14631</v>
       </c>
@@ -951,6 +1094,12 @@
       </c>
       <c r="H15" t="s">
         <v>11</v>
+      </c>
+      <c r="I15" t="s">
+        <v>34</v>
+      </c>
+      <c r="J15" t="s">
+        <v>40</v>
       </c>
       <c r="K15" t="s">
         <v>27</v>
@@ -972,6 +1121,9 @@
       <c r="D16">
         <v>0.39400000000000002</v>
       </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
       <c r="F16" s="2">
         <v>14293</v>
       </c>
@@ -983,6 +1135,9 @@
       </c>
       <c r="I16" t="s">
         <v>32</v>
+      </c>
+      <c r="J16" t="s">
+        <v>35</v>
       </c>
       <c r="K16" t="s">
         <v>27</v>
@@ -1001,6 +1156,12 @@
       <c r="C17">
         <v>0.51</v>
       </c>
+      <c r="D17">
+        <v>0.38600000000000001</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
       <c r="F17" s="2">
         <v>13925</v>
       </c>
@@ -1009,6 +1170,9 @@
       </c>
       <c r="H17" t="s">
         <v>11</v>
+      </c>
+      <c r="J17" t="s">
+        <v>35</v>
       </c>
       <c r="K17" t="s">
         <v>27</v>
@@ -1030,6 +1194,9 @@
       <c r="D18">
         <v>0.51800000000000002</v>
       </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
       <c r="F18" s="2">
         <v>14101</v>
       </c>
@@ -1041,6 +1208,9 @@
       </c>
       <c r="I18" t="s">
         <v>25</v>
+      </c>
+      <c r="J18" t="s">
+        <v>35</v>
       </c>
       <c r="K18" t="s">
         <v>27</v>
@@ -1062,6 +1232,9 @@
       <c r="D19">
         <v>0.51539999999999997</v>
       </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
       <c r="F19" s="2">
         <v>18923</v>
       </c>
@@ -1073,6 +1246,9 @@
       </c>
       <c r="I19" t="s">
         <v>30</v>
+      </c>
+      <c r="J19" t="s">
+        <v>35</v>
       </c>
       <c r="K19" t="s">
         <v>27</v>
@@ -1094,6 +1270,9 @@
       <c r="D20" s="3">
         <v>0.40439999999999998</v>
       </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
       <c r="F20" s="2">
         <v>19929</v>
       </c>
@@ -1105,6 +1284,9 @@
       </c>
       <c r="I20" t="s">
         <v>29</v>
+      </c>
+      <c r="J20" t="s">
+        <v>35</v>
       </c>
       <c r="K20" t="s">
         <v>27</v>
@@ -1126,6 +1308,9 @@
       <c r="D21">
         <v>0.4476</v>
       </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
       <c r="F21" s="2">
         <v>18687</v>
       </c>
@@ -1137,6 +1322,9 @@
       </c>
       <c r="I21" t="s">
         <v>28</v>
+      </c>
+      <c r="J21" t="s">
+        <v>35</v>
       </c>
       <c r="K21" t="s">
         <v>27</v>
@@ -1155,6 +1343,12 @@
       <c r="C22">
         <v>0.54479999999999995</v>
       </c>
+      <c r="D22">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
       <c r="F22" s="2">
         <v>19952</v>
       </c>
@@ -1163,6 +1357,9 @@
       </c>
       <c r="H22" t="s">
         <v>11</v>
+      </c>
+      <c r="J22" t="s">
+        <v>35</v>
       </c>
       <c r="K22" t="s">
         <v>27</v>
@@ -1181,6 +1378,12 @@
       <c r="C23">
         <v>0.55010000000000003</v>
       </c>
+      <c r="D23">
+        <v>0.41799999999999998</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
       <c r="F23" s="2">
         <v>20732</v>
       </c>
@@ -1189,6 +1392,9 @@
       </c>
       <c r="H23" t="s">
         <v>11</v>
+      </c>
+      <c r="J23" t="s">
+        <v>35</v>
       </c>
       <c r="K23" t="s">
         <v>17</v>
@@ -1210,6 +1416,9 @@
       <c r="D24">
         <v>0.79390000000000005</v>
       </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
       <c r="F24" s="2">
         <v>12206</v>
       </c>
@@ -1221,6 +1430,9 @@
       </c>
       <c r="I24" t="s">
         <v>31</v>
+      </c>
+      <c r="J24" t="s">
+        <v>39</v>
       </c>
       <c r="K24" t="s">
         <v>27</v>
@@ -1239,6 +1451,12 @@
       <c r="C25">
         <v>0.40139999999999998</v>
       </c>
+      <c r="D25">
+        <v>0.77859999999999996</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
       <c r="F25" s="2">
         <v>12344</v>
       </c>
@@ -1247,6 +1465,12 @@
       </c>
       <c r="H25" t="s">
         <v>11</v>
+      </c>
+      <c r="I25" t="s">
+        <v>33</v>
+      </c>
+      <c r="J25" t="s">
+        <v>39</v>
       </c>
       <c r="K25" t="s">
         <v>27</v>
@@ -1265,6 +1489,12 @@
       <c r="C26">
         <v>0.40250000000000002</v>
       </c>
+      <c r="D26">
+        <v>0.74129999999999996</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
       <c r="F26" s="2">
         <v>14631</v>
       </c>
@@ -1273,6 +1503,12 @@
       </c>
       <c r="H26" t="s">
         <v>11</v>
+      </c>
+      <c r="I26" t="s">
+        <v>34</v>
+      </c>
+      <c r="J26" t="s">
+        <v>41</v>
       </c>
       <c r="K26" t="s">
         <v>27</v>
@@ -1294,6 +1530,9 @@
       <c r="D27">
         <v>0.753</v>
       </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
       <c r="F27" s="2">
         <v>14293</v>
       </c>
@@ -1305,6 +1544,9 @@
       </c>
       <c r="I27" t="s">
         <v>32</v>
+      </c>
+      <c r="J27" t="s">
+        <v>35</v>
       </c>
       <c r="K27" t="s">
         <v>27</v>
@@ -1323,6 +1565,12 @@
       <c r="C28">
         <v>0.40360000000000001</v>
       </c>
+      <c r="D28">
+        <v>0.72599999999999998</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
       <c r="F28" s="2">
         <v>13925</v>
       </c>
@@ -1331,6 +1579,9 @@
       </c>
       <c r="H28" t="s">
         <v>11</v>
+      </c>
+      <c r="J28" t="s">
+        <v>35</v>
       </c>
       <c r="K28" t="s">
         <v>27</v>
@@ -1352,6 +1603,9 @@
       <c r="D29">
         <v>1.0489999999999999</v>
       </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
       <c r="F29" s="2">
         <v>14101</v>
       </c>
@@ -1363,6 +1617,9 @@
       </c>
       <c r="I29" t="s">
         <v>25</v>
+      </c>
+      <c r="J29" t="s">
+        <v>35</v>
       </c>
       <c r="K29" t="s">
         <v>27</v>
@@ -1384,6 +1641,9 @@
       <c r="D30">
         <v>0.70250000000000001</v>
       </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
       <c r="F30" s="2">
         <v>18923</v>
       </c>
@@ -1395,6 +1655,9 @@
       </c>
       <c r="I30" t="s">
         <v>30</v>
+      </c>
+      <c r="J30" t="s">
+        <v>35</v>
       </c>
       <c r="K30" t="s">
         <v>27</v>
@@ -1416,6 +1679,9 @@
       <c r="D31" s="3">
         <v>0.68489999999999995</v>
       </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
       <c r="F31" s="2">
         <v>19929</v>
       </c>
@@ -1427,6 +1693,9 @@
       </c>
       <c r="I31" t="s">
         <v>29</v>
+      </c>
+      <c r="J31" t="s">
+        <v>35</v>
       </c>
       <c r="K31" t="s">
         <v>27</v>
@@ -1448,6 +1717,9 @@
       <c r="D32">
         <v>0.64790000000000003</v>
       </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
       <c r="F32" s="2">
         <v>18687</v>
       </c>
@@ -1459,6 +1731,9 @@
       </c>
       <c r="I32" t="s">
         <v>28</v>
+      </c>
+      <c r="J32" t="s">
+        <v>35</v>
       </c>
       <c r="K32" t="s">
         <v>27</v>
@@ -1477,6 +1752,12 @@
       <c r="C33">
         <v>0.40429999999999999</v>
       </c>
+      <c r="D33">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
       <c r="F33" s="2">
         <v>19952</v>
       </c>
@@ -1485,6 +1766,9 @@
       </c>
       <c r="H33" t="s">
         <v>11</v>
+      </c>
+      <c r="J33" t="s">
+        <v>35</v>
       </c>
       <c r="K33" t="s">
         <v>27</v>
@@ -1503,6 +1787,12 @@
       <c r="C34">
         <v>0.40400000000000003</v>
       </c>
+      <c r="D34">
+        <v>0.628</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
       <c r="F34" s="2">
         <v>20732</v>
       </c>
@@ -1511,6 +1801,9 @@
       </c>
       <c r="H34" t="s">
         <v>11</v>
+      </c>
+      <c r="J34" t="s">
+        <v>36</v>
       </c>
       <c r="K34" t="s">
         <v>17</v>
@@ -1532,6 +1825,9 @@
       <c r="D35">
         <v>0.81159999999999999</v>
       </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
       <c r="F35" s="2">
         <v>12206</v>
       </c>
@@ -1543,6 +1839,9 @@
       </c>
       <c r="I35" t="s">
         <v>31</v>
+      </c>
+      <c r="J35" t="s">
+        <v>37</v>
       </c>
       <c r="K35" t="s">
         <v>27</v>
@@ -1561,6 +1860,12 @@
       <c r="C36">
         <v>0.76</v>
       </c>
+      <c r="D36">
+        <v>0.80269999999999997</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
       <c r="F36" s="2">
         <v>12344</v>
       </c>
@@ -1569,6 +1874,12 @@
       </c>
       <c r="H36" t="s">
         <v>11</v>
+      </c>
+      <c r="I36" t="s">
+        <v>33</v>
+      </c>
+      <c r="J36" t="s">
+        <v>37</v>
       </c>
       <c r="K36" t="s">
         <v>27</v>
@@ -1587,6 +1898,12 @@
       <c r="C37">
         <v>0.74250000000000005</v>
       </c>
+      <c r="D37">
+        <v>0.78449999999999998</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
       <c r="F37" s="2">
         <v>14631</v>
       </c>
@@ -1595,6 +1912,12 @@
       </c>
       <c r="H37" t="s">
         <v>11</v>
+      </c>
+      <c r="I37" t="s">
+        <v>34</v>
+      </c>
+      <c r="J37" t="s">
+        <v>37</v>
       </c>
       <c r="K37" t="s">
         <v>27</v>
@@ -1616,6 +1939,9 @@
       <c r="D38">
         <v>0.79100000000000004</v>
       </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
       <c r="F38" s="2">
         <v>14293</v>
       </c>
@@ -1627,6 +1953,9 @@
       </c>
       <c r="I38" t="s">
         <v>32</v>
+      </c>
+      <c r="J38" t="s">
+        <v>37</v>
       </c>
       <c r="K38" t="s">
         <v>27</v>
@@ -1645,6 +1974,12 @@
       <c r="C39">
         <v>0.62</v>
       </c>
+      <c r="D39">
+        <v>0.77300000000000002</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
       <c r="F39" s="2">
         <v>13925</v>
       </c>
@@ -1653,6 +1988,9 @@
       </c>
       <c r="H39" t="s">
         <v>11</v>
+      </c>
+      <c r="J39" t="s">
+        <v>37</v>
       </c>
       <c r="K39" t="s">
         <v>27</v>
@@ -1674,6 +2012,9 @@
       <c r="D40">
         <v>0.75600000000000001</v>
       </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
       <c r="F40" s="2">
         <v>14101</v>
       </c>
@@ -1685,6 +2026,9 @@
       </c>
       <c r="I40" t="s">
         <v>25</v>
+      </c>
+      <c r="J40" t="s">
+        <v>37</v>
       </c>
       <c r="K40" t="s">
         <v>27</v>
@@ -1706,6 +2050,9 @@
       <c r="D41">
         <v>0.63690000000000002</v>
       </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
       <c r="F41" s="2">
         <v>18923</v>
       </c>
@@ -1717,6 +2064,9 @@
       </c>
       <c r="I41" t="s">
         <v>30</v>
+      </c>
+      <c r="J41" t="s">
+        <v>37</v>
       </c>
       <c r="K41" t="s">
         <v>27</v>
@@ -1738,6 +2088,9 @@
       <c r="D42" s="3">
         <v>0.60580000000000001</v>
       </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
       <c r="F42" s="2">
         <v>19929</v>
       </c>
@@ -1749,6 +2102,9 @@
       </c>
       <c r="I42" t="s">
         <v>29</v>
+      </c>
+      <c r="J42" t="s">
+        <v>37</v>
       </c>
       <c r="K42" t="s">
         <v>27</v>
@@ -1770,6 +2126,9 @@
       <c r="D43">
         <v>0.5897</v>
       </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
       <c r="F43" s="2">
         <v>18687</v>
       </c>
@@ -1781,6 +2140,9 @@
       </c>
       <c r="I43" t="s">
         <v>28</v>
+      </c>
+      <c r="J43" t="s">
+        <v>37</v>
       </c>
       <c r="K43" t="s">
         <v>27</v>
@@ -1799,6 +2161,12 @@
       <c r="C44">
         <v>0.6</v>
       </c>
+      <c r="D44">
+        <v>0.57499999999999996</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
       <c r="F44" s="2">
         <v>19952</v>
       </c>
@@ -1807,6 +2175,9 @@
       </c>
       <c r="H44" t="s">
         <v>11</v>
+      </c>
+      <c r="J44" t="s">
+        <v>37</v>
       </c>
       <c r="K44" t="s">
         <v>27</v>
@@ -1825,6 +2196,12 @@
       <c r="C45">
         <v>0.6</v>
       </c>
+      <c r="D45">
+        <v>0.57199999999999995</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
       <c r="F45" s="2">
         <v>20732</v>
       </c>
@@ -1833,6 +2210,9 @@
       </c>
       <c r="H45" t="s">
         <v>11</v>
+      </c>
+      <c r="J45" t="s">
+        <v>37</v>
       </c>
       <c r="K45" t="s">
         <v>17</v>
@@ -1854,6 +2234,9 @@
       <c r="D46">
         <v>0.85550000000000004</v>
       </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
       <c r="F46" s="2">
         <v>12206</v>
       </c>
@@ -1865,6 +2248,9 @@
       </c>
       <c r="I46" t="s">
         <v>31</v>
+      </c>
+      <c r="J46" t="s">
+        <v>37</v>
       </c>
       <c r="K46" t="s">
         <v>27</v>
@@ -1883,6 +2269,12 @@
       <c r="C47">
         <v>0.77</v>
       </c>
+      <c r="D47">
+        <v>0.85929999999999995</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
       <c r="F47" s="2">
         <v>12344</v>
       </c>
@@ -1891,6 +2283,12 @@
       </c>
       <c r="H47" t="s">
         <v>11</v>
+      </c>
+      <c r="I47" t="s">
+        <v>33</v>
+      </c>
+      <c r="J47" t="s">
+        <v>37</v>
       </c>
       <c r="K47" t="s">
         <v>27</v>
@@ -1909,6 +2307,12 @@
       <c r="C48">
         <v>0.77</v>
       </c>
+      <c r="D48">
+        <v>0.84209999999999996</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
       <c r="F48" s="2">
         <v>14631</v>
       </c>
@@ -1917,6 +2321,12 @@
       </c>
       <c r="H48" t="s">
         <v>11</v>
+      </c>
+      <c r="I48" t="s">
+        <v>34</v>
+      </c>
+      <c r="J48" t="s">
+        <v>37</v>
       </c>
       <c r="K48" t="s">
         <v>27</v>
@@ -1938,6 +2348,9 @@
       <c r="D49">
         <v>0.86099999999999999</v>
       </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
       <c r="F49" s="2">
         <v>14293</v>
       </c>
@@ -1949,6 +2362,9 @@
       </c>
       <c r="I49" t="s">
         <v>32</v>
+      </c>
+      <c r="J49" t="s">
+        <v>37</v>
       </c>
       <c r="K49" t="s">
         <v>27</v>
@@ -1967,6 +2383,12 @@
       <c r="C50">
         <v>0.625</v>
       </c>
+      <c r="D50">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
       <c r="F50" s="2">
         <v>13925</v>
       </c>
@@ -1975,6 +2397,9 @@
       </c>
       <c r="H50" t="s">
         <v>11</v>
+      </c>
+      <c r="J50" t="s">
+        <v>37</v>
       </c>
       <c r="K50" t="s">
         <v>27</v>
@@ -1996,6 +2421,9 @@
       <c r="D51">
         <v>0.78500000000000003</v>
       </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
       <c r="F51" s="2">
         <v>14101</v>
       </c>
@@ -2007,6 +2435,9 @@
       </c>
       <c r="I51" t="s">
         <v>25</v>
+      </c>
+      <c r="J51" t="s">
+        <v>37</v>
       </c>
       <c r="K51" t="s">
         <v>27</v>
@@ -2028,6 +2459,9 @@
       <c r="D52">
         <v>0.68379999999999996</v>
       </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
       <c r="F52" s="2">
         <v>18923</v>
       </c>
@@ -2039,6 +2473,9 @@
       </c>
       <c r="I52" t="s">
         <v>30</v>
+      </c>
+      <c r="J52" t="s">
+        <v>37</v>
       </c>
       <c r="K52" t="s">
         <v>27</v>
@@ -2060,6 +2497,9 @@
       <c r="D53" s="3">
         <v>0.64100000000000001</v>
       </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
       <c r="F53" s="2">
         <v>19929</v>
       </c>
@@ -2071,6 +2511,9 @@
       </c>
       <c r="I53" t="s">
         <v>29</v>
+      </c>
+      <c r="J53" t="s">
+        <v>37</v>
       </c>
       <c r="K53" t="s">
         <v>27</v>
@@ -2092,6 +2535,9 @@
       <c r="D54">
         <v>0.61909999999999998</v>
       </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
       <c r="F54" s="2">
         <v>18687</v>
       </c>
@@ -2103,6 +2549,9 @@
       </c>
       <c r="I54" t="s">
         <v>28</v>
+      </c>
+      <c r="J54" t="s">
+        <v>37</v>
       </c>
       <c r="K54" t="s">
         <v>27</v>
@@ -2121,6 +2570,12 @@
       <c r="C55">
         <v>0.75080000000000002</v>
       </c>
+      <c r="D55">
+        <v>0.60799999999999998</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
       <c r="F55" s="2">
         <v>19952</v>
       </c>
@@ -2129,6 +2584,9 @@
       </c>
       <c r="H55" t="s">
         <v>11</v>
+      </c>
+      <c r="J55" t="s">
+        <v>37</v>
       </c>
       <c r="K55" t="s">
         <v>27</v>
@@ -2147,6 +2605,12 @@
       <c r="C56">
         <v>0.75</v>
       </c>
+      <c r="D56">
+        <v>0.60499999999999998</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
       <c r="F56" s="2">
         <v>20732</v>
       </c>
@@ -2155,6 +2619,9 @@
       </c>
       <c r="H56" t="s">
         <v>11</v>
+      </c>
+      <c r="J56" t="s">
+        <v>37</v>
       </c>
       <c r="K56" t="s">
         <v>17</v>

</xml_diff>